<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-19 14:22:53)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -18263,7 +18263,7 @@
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>26-04</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X144" t="inlineStr">
@@ -18278,12 +18278,12 @@
       </c>
       <c r="Z144" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA144" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>19.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 09:01:45)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB564"/>
+  <dimension ref="A1:AB565"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53594,6 +53594,109 @@
         </is>
       </c>
     </row>
+    <row r="565">
+      <c r="A565" t="n">
+        <v>564</v>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Temirova Yulduzxon</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr"/>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>20.10.2026</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>Luxmon qizi</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Temirova Yulduzxon Luxmon qizi</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>AD1646787</t>
+        </is>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>40307912640022</t>
+        </is>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>11.08.2022</t>
+        </is>
+      </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>03.07.1991</t>
+        </is>
+      </c>
+      <c r="N565" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O565" t="inlineStr">
+        <is>
+          <t>K 1611606</t>
+        </is>
+      </c>
+      <c r="P565" t="inlineStr"/>
+      <c r="Q565" t="inlineStr">
+        <is>
+          <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R565" t="inlineStr">
+        <is>
+          <t>Diplom</t>
+        </is>
+      </c>
+      <c r="S565" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="T565" t="inlineStr"/>
+      <c r="U565" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W565" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y565" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB565" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 09:31:50)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -53613,7 +53613,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E565" t="inlineStr"/>
       <c r="F565" t="inlineStr">
         <is>
           <t>20.10.2026</t>
@@ -53659,7 +53658,6 @@
           <t>K 1611606</t>
         </is>
       </c>
-      <c r="P565" t="inlineStr"/>
       <c r="Q565" t="inlineStr">
         <is>
           <t>Kitob qishloq xo'jalik kasb-hunar kolleji</t>
@@ -53675,7 +53673,6 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="T565" t="inlineStr"/>
       <c r="U565" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -53693,7 +53690,7 @@
       </c>
       <c r="AB565" t="inlineStr">
         <is>
-          <t>KIRITILDI</t>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 09:47:51)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -22903,6 +22903,11 @@
           <t>26-02</t>
         </is>
       </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
       <c r="Z182" t="inlineStr">
         <is>
           <t>T-40/2</t>
@@ -22911,6 +22916,11 @@
       <c r="AA182" t="inlineStr">
         <is>
           <t>02.09.2026</t>
+        </is>
+      </c>
+      <c r="AB182" t="inlineStr">
+        <is>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 09:48:24)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -17520,7 +17520,7 @@
       </c>
       <c r="Y138" t="inlineStr">
         <is>
-          <t>TASDIQLANDI</t>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
       <c r="Z138" t="inlineStr">
@@ -17531,6 +17531,11 @@
       <c r="AA138" t="inlineStr">
         <is>
           <t>02.09.2026</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 10:39:40)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB565"/>
+  <dimension ref="A1:AB566"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53709,6 +53709,109 @@
         </is>
       </c>
     </row>
+    <row r="566">
+      <c r="A566" t="n">
+        <v>565</v>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Karimova Umida</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr"/>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>20.10.2026</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>Dusmurod qizi</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Karimova Umida Dusmurod qizi</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>AE7890316</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>60811065680047</t>
+        </is>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>07.07.2026</t>
+        </is>
+      </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>08.11.2006</t>
+        </is>
+      </c>
+      <c r="N566" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O566" t="inlineStr">
+        <is>
+          <t>UM 02314713</t>
+        </is>
+      </c>
+      <c r="P566" t="inlineStr"/>
+      <c r="Q566" t="inlineStr">
+        <is>
+          <t>301-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R566" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S566" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T566" t="inlineStr"/>
+      <c r="U566" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W566" t="inlineStr">
+        <is>
+          <t>24-13</t>
+        </is>
+      </c>
+      <c r="Y566" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB566" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 10:40:30)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -53728,7 +53728,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E566" t="inlineStr"/>
       <c r="F566" t="inlineStr">
         <is>
           <t>20.10.2026</t>
@@ -53774,7 +53773,6 @@
           <t>UM 02314713</t>
         </is>
       </c>
-      <c r="P566" t="inlineStr"/>
       <c r="Q566" t="inlineStr">
         <is>
           <t>301-sonli umumiy o'rta ta'lim maktabini</t>
@@ -53790,7 +53788,6 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="T566" t="inlineStr"/>
       <c r="U566" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -53808,7 +53805,7 @@
       </c>
       <c r="AB566" t="inlineStr">
         <is>
-          <t>KIRITILDI</t>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-21 08:59:00)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB566"/>
+  <dimension ref="A1:AB567"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53809,6 +53809,109 @@
         </is>
       </c>
     </row>
+    <row r="567">
+      <c r="A567" t="n">
+        <v>566</v>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Xayrullayeva Asila</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Farmatsiya ishi</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr"/>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>21.10.2026</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>Azamat qizi</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Xayrullayeva Asila Azamat qizi</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>AE6045063</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>62103095680022</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>26.01.2026</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>21.03.2009</t>
+        </is>
+      </c>
+      <c r="N567" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>UM 03728305</t>
+        </is>
+      </c>
+      <c r="P567" t="inlineStr"/>
+      <c r="Q567" t="inlineStr">
+        <is>
+          <t>Kitob tumani 9-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="R567" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T567" t="inlineStr"/>
+      <c r="U567" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W567" t="inlineStr">
+        <is>
+          <t>26-01</t>
+        </is>
+      </c>
+      <c r="Y567" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB567" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-22 09:41:48)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -17510,7 +17510,7 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X138" t="inlineStr">
@@ -17525,12 +17525,12 @@
       </c>
       <c r="Z138" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA138" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="AB138" t="inlineStr">
@@ -53828,7 +53828,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E567" t="inlineStr"/>
       <c r="F567" t="inlineStr">
         <is>
           <t>21.10.2026</t>
@@ -53874,7 +53873,6 @@
           <t>UM 03728305</t>
         </is>
       </c>
-      <c r="P567" t="inlineStr"/>
       <c r="Q567" t="inlineStr">
         <is>
           <t>Kitob tumani 9-sonli umumiy o'rta ta'lim maktabi</t>
@@ -53890,7 +53888,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T567" t="inlineStr"/>
       <c r="U567" t="inlineStr">
         <is>
           <t>TOPILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-22 09:43:06)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -10462,7 +10462,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
@@ -10477,12 +10477,12 @@
       </c>
       <c r="Z81" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
     </row>
@@ -18994,7 +18994,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="X150" t="inlineStr">
@@ -19009,12 +19009,12 @@
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(direction): 01-guruh faqat Farmatsiya ishi, qolgan barcha guruhlar Hamshiralik ishi qilib bazalar va ma'lumotnoma to'g'rilandi
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Farmatsiya ishi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -826,6 +826,11 @@
           <t>Abdixalilova Shohzoda</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -956,6 +961,11 @@
           <t>Abdixoliqova Elmira</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>286</t>
@@ -1083,7 +1093,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1213,7 +1223,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Farmatsiya ishi</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1343,7 +1353,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Feldsherlik ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1473,7 +1483,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1603,7 +1613,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1968,7 +1978,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2093,7 +2103,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2463,7 +2473,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Feldsherlik ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2593,7 +2603,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2723,7 +2733,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2853,7 +2863,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2978,7 +2988,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3096,6 +3106,11 @@
           <t>Davlatova Gulnoza</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -3219,7 +3234,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -3344,7 +3359,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Farmatsiya ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3469,7 +3484,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3589,7 +3604,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3719,7 +3734,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3834,7 +3849,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3962,6 +3977,11 @@
           <t>Eshquvatova Yulduz</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>267</t>
@@ -4075,7 +4095,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4200,7 +4220,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -4318,7 +4338,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4448,7 +4468,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4578,7 +4598,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4673,7 +4693,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4799,6 +4819,11 @@
           <t>Hamroqulova Farzona</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>278</t>
@@ -4919,6 +4944,11 @@
           <t>Hamroqulova Marjona</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -5051,7 +5081,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5171,7 +5201,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5431,7 +5461,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5561,7 +5591,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Farmatsiya ishi</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5684,6 +5714,11 @@
           <t>Ibragimova Gulnoza</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>308</t>
@@ -5934,7 +5969,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -6064,7 +6099,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6194,7 +6229,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -6299,7 +6334,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -6429,7 +6464,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -6559,7 +6594,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6689,7 +6724,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Feldsherlik ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6934,7 +6969,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7064,7 +7099,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7194,7 +7229,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7324,7 +7359,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -7444,7 +7479,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7577,6 +7612,11 @@
           <t>Karimova Nozliya</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -7814,7 +7854,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7944,7 +7984,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -8074,7 +8114,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -8177,6 +8217,11 @@
           <t>Mahmudova Gulsanam</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -8302,7 +8347,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -8552,7 +8597,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -8680,6 +8725,11 @@
           <t>Mansurova Gulasal</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -8793,6 +8843,11 @@
           <t>Maxmarajabova Zerda</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
           <t>253</t>
@@ -8915,7 +8970,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -9045,7 +9100,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -9178,7 +9233,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -9308,7 +9363,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi</t>
+          <t>Farmatsiya ishi</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -9438,7 +9493,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -9616,7 +9671,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -9746,7 +9801,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -9871,7 +9926,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -10126,7 +10181,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -10374,7 +10429,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -10497,7 +10552,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -10627,7 +10682,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -10743,6 +10798,11 @@
           <t>Nafasova Sevinch</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
           <t>266</t>
@@ -10863,7 +10923,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -11433,7 +11493,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -11563,7 +11623,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -11683,7 +11743,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Farmatsiya ishi</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -11813,7 +11873,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -11943,7 +12003,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -12073,7 +12133,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -12208,7 +12268,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -12428,7 +12488,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -12551,6 +12611,11 @@
           <t>Ozodova Klara</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>285</t>
@@ -12671,7 +12736,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -12801,7 +12866,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -12931,7 +12996,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -13176,7 +13241,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -13436,7 +13501,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -13556,7 +13621,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -13691,7 +13756,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -14066,7 +14131,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Farmatsiya ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -14191,7 +14256,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -14319,7 +14384,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -14444,7 +14509,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -14544,7 +14609,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -14924,7 +14989,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -15042,6 +15107,11 @@
           <t>Saydalimova Ruxshona</t>
         </is>
       </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D119" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -15172,6 +15242,11 @@
           <t>Sayfillayeva Shodiyona</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D120" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -15304,7 +15379,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -15427,6 +15502,11 @@
           <t>Sayidova Dilafro'z</t>
         </is>
       </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>263</t>
@@ -15549,7 +15629,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -15679,7 +15759,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -15809,7 +15889,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -15939,7 +16019,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -16177,6 +16257,11 @@
           <t>Suyarova Dinora</t>
         </is>
       </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>306</t>
@@ -16295,7 +16380,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -16420,7 +16505,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -16668,6 +16753,11 @@
           <t>To'raboyeva Sabrina</t>
         </is>
       </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -16795,7 +16885,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -16920,7 +17010,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -17045,7 +17135,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -17175,7 +17265,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -17293,6 +17383,11 @@
           <t>Turayeva Dilsuz</t>
         </is>
       </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Farmatsiya ishi</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
           <t>268</t>
@@ -17415,7 +17510,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 2 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -17675,7 +17770,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Feldsherlik ishi</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -17798,6 +17893,11 @@
           <t>Tursunova Aziza</t>
         </is>
       </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="D141" t="inlineStr">
         <is>
           <t>To'lov qildi</t>
@@ -17925,7 +18025,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -18050,7 +18150,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -18303,7 +18403,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -18408,7 +18508,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -18536,6 +18636,11 @@
           <t>Umirova Sevinch</t>
         </is>
       </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>298</t>
@@ -18651,7 +18756,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -19029,7 +19134,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -19159,7 +19264,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -19284,7 +19389,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -19413,7 +19518,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -19521,7 +19626,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -19651,7 +19756,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -19776,7 +19881,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -19904,7 +20009,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -20034,7 +20139,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -20164,7 +20269,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -20297,7 +20402,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -20422,7 +20527,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -20527,7 +20632,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -20657,7 +20762,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -20780,7 +20885,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -20910,7 +21015,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -21040,7 +21145,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -21175,7 +21280,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -21300,7 +21405,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -21430,7 +21535,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -21560,7 +21665,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -21690,7 +21795,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -21945,7 +22050,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -22070,7 +22175,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -22200,7 +22305,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -22315,7 +22420,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -22420,7 +22525,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -22525,7 +22630,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -22630,7 +22735,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -22740,7 +22845,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -22835,7 +22940,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -22940,7 +23045,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -23045,7 +23150,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -53175,7 +53280,7 @@
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
@@ -53290,7 +53395,7 @@
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
@@ -53400,7 +53505,7 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
@@ -53515,7 +53620,7 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
@@ -53620,7 +53725,7 @@
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
@@ -53720,7 +53825,7 @@
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
+          <t>Hamshiralik ishi</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-23 14:44:05)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -49985,12 +49985,22 @@
       </c>
       <c r="W520" t="inlineStr">
         <is>
-          <t>25-22</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y520" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z520" t="inlineStr">
+        <is>
+          <t>T-58</t>
+        </is>
+      </c>
+      <c r="AA520" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-23 14:45:23)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -31460,12 +31460,22 @@
       </c>
       <c r="W288" t="inlineStr">
         <is>
-          <t>24-11</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y288" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z288" t="inlineStr">
+        <is>
+          <t>t-59</t>
+        </is>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-23 15:56:37)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB567"/>
+  <dimension ref="A1:AB568"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54034,6 +54034,117 @@
         </is>
       </c>
     </row>
+    <row r="568">
+      <c r="A568" t="n">
+        <v>567</v>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Xurramova Nilufar</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>334</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Murodulla qizi</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Xurramova Nilufar Murodulla qizi</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>AE2166628</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>62603085590057</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>03.04.2025</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>26.03.2008</t>
+        </is>
+      </c>
+      <c r="N568" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>UM 03754800</t>
+        </is>
+      </c>
+      <c r="P568" t="inlineStr"/>
+      <c r="Q568" t="inlineStr">
+        <is>
+          <t>43-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="R568" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S568" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T568" t="inlineStr">
+        <is>
+          <t>887202608</t>
+        </is>
+      </c>
+      <c r="U568" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W568" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y568" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB568" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-23 15:58:34)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB568"/>
+  <dimension ref="A1:AB569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54103,7 +54103,6 @@
           <t>UM 03754800</t>
         </is>
       </c>
-      <c r="P568" t="inlineStr"/>
       <c r="Q568" t="inlineStr">
         <is>
           <t>43-sonli umumiy o'rta ta'lim maktabi</t>
@@ -54140,6 +54139,109 @@
         </is>
       </c>
       <c r="AB568" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="n">
+        <v>568</v>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Uralova Jasmina</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr"/>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Anvarxon qizi</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Uralova Jasmina Anvarxon qizi</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>AD8707337</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>60302075590065</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>20.09.2024</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>03.02.2007</t>
+        </is>
+      </c>
+      <c r="N569" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>UM 03295750</t>
+        </is>
+      </c>
+      <c r="P569" t="inlineStr"/>
+      <c r="Q569" t="inlineStr">
+        <is>
+          <t>7-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R569" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S569" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T569" t="inlineStr"/>
+      <c r="U569" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W569" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y569" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB569" t="inlineStr">
         <is>
           <t>KIRITILDI</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-23 15:59:18)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -23030,7 +23030,7 @@
       </c>
       <c r="AB182" t="inlineStr">
         <is>
-          <t>KIRITILMAGAN</t>
+          <t>KIRITILDI</t>
         </is>
       </c>
     </row>
@@ -54140,7 +54140,7 @@
       </c>
       <c r="AB568" t="inlineStr">
         <is>
-          <t>KIRITILDI</t>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>
@@ -54163,7 +54163,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E569" t="inlineStr"/>
       <c r="F569" t="inlineStr">
         <is>
           <t>23.10.2026</t>
@@ -54209,7 +54208,6 @@
           <t>UM 03295750</t>
         </is>
       </c>
-      <c r="P569" t="inlineStr"/>
       <c r="Q569" t="inlineStr">
         <is>
           <t>7-sonli umumiy o'rta ta'lim maktabini</t>
@@ -54225,7 +54223,6 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="T569" t="inlineStr"/>
       <c r="U569" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -54238,12 +54235,12 @@
       </c>
       <c r="Y569" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="AB569" t="inlineStr">
         <is>
-          <t>KIRITILDI</t>
+          <t>KIRITILMAGAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-26 12:11:53)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -49995,7 +49995,7 @@
       </c>
       <c r="W520" t="inlineStr">
         <is>
-          <t>Akademik ta'til olganlar</t>
+          <t>25-22</t>
         </is>
       </c>
       <c r="Y520" t="inlineStr">
@@ -50003,11 +50003,7 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z520" t="inlineStr">
-        <is>
-          <t>T-58</t>
-        </is>
-      </c>
+      <c r="Z520" t="inlineStr"/>
       <c r="AA520" t="inlineStr">
         <is>
           <t>23.10.2026</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-27 09:00:50)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB569"/>
+  <dimension ref="A1:AB570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50003,7 +50003,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z520" t="inlineStr"/>
       <c r="AA520" t="inlineStr">
         <is>
           <t>23.10.2026</t>
@@ -54237,6 +54236,109 @@
       <c r="AB569" t="inlineStr">
         <is>
           <t>KIRITILMAGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="n">
+        <v>569</v>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Chorshanova Safiya</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr"/>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Ibodullo qizi</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Chorshanova Safiya Ibodullo qizi</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>AE3818237</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>61001095680039</t>
+        </is>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>18.08.2025</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>10.01.2009</t>
+        </is>
+      </c>
+      <c r="N570" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O570" t="inlineStr">
+        <is>
+          <t>UM 03728107</t>
+        </is>
+      </c>
+      <c r="P570" t="inlineStr"/>
+      <c r="Q570" t="inlineStr">
+        <is>
+          <t>5-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R570" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S570" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T570" t="inlineStr"/>
+      <c r="U570" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W570" t="inlineStr">
+        <is>
+          <t>26-04</t>
+        </is>
+      </c>
+      <c r="Y570" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB570" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-28 17:02:31)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -53815,12 +53815,22 @@
       </c>
       <c r="W565" t="inlineStr">
         <is>
-          <t>26-03</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y565" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z565" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="AA565" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="AB565" t="inlineStr">
@@ -54258,7 +54268,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E570" t="inlineStr"/>
       <c r="F570" t="inlineStr">
         <is>
           <t>27.10.2026</t>
@@ -54304,7 +54313,6 @@
           <t>UM 03728107</t>
         </is>
       </c>
-      <c r="P570" t="inlineStr"/>
       <c r="Q570" t="inlineStr">
         <is>
           <t>5-sonli umumiy o'rta ta'lim maktabini</t>
@@ -54320,7 +54328,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T570" t="inlineStr"/>
       <c r="U570" t="inlineStr">
         <is>
           <t>TOPILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-29 16:21:00)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -8189,7 +8189,7 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
@@ -8199,12 +8199,12 @@
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>29.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>